<commit_message>
Task 1: update ceramics quote with real data (set 4 cups+4 plates, Lizeth, restaurant venue)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
@@ -80,7 +80,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00Efe6d5"/>
+        <fgColor rgb="00EFE6D5"/>
       </patternFill>
     </fill>
   </fills>
@@ -110,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -118,12 +118,18 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -216,49 +222,39 @@
     <author>Alado</author>
   </authors>
   <commentList>
-    <comment ref="B9" authorId="0" shapeId="0">
+    <comment ref="B10" authorId="0" shapeId="0">
       <text>
-        <t>Markup sobre el costo. 45% es un margen sano para taller-experiencia.</t>
+        <t>0% si es transferencia/efectivo.</t>
       </text>
     </comment>
-    <comment ref="B10" authorId="0" shapeId="0">
+    <comment ref="B20" authorId="0" shapeId="0">
       <text>
-        <t>Si cobras por link/online (~3–4%). Pon 0% si es transferencia/efectivo.</t>
+        <t>ESTIMADO — confirmar costo real de pigmentos/esmaltes por persona.</t>
       </text>
     </comment>
-    <comment ref="B14" authorId="0" shapeId="0">
+    <comment ref="B21" authorId="0" shapeId="0">
       <text>
-        <t>Taza/plato/pieza mediana en blanco.</t>
+        <t>ESTIMADO — pon $0 si Alado tiene horno propio; o el costo real de cocción del set.</t>
       </text>
     </comment>
-    <comment ref="B15" authorId="0" shapeId="0">
+    <comment ref="B29" authorId="0" shapeId="0">
       <text>
-        <t>Prorrateado por persona.</t>
+        <t>Son los fundadores. Pon un valor si quieres imputar su tiempo; 0 si no.</t>
       </text>
     </comment>
-    <comment ref="B16" authorId="0" shapeId="0">
+    <comment ref="B30" authorId="0" shapeId="0">
       <text>
-        <t>Cocción (tercerizada o propia).</t>
+        <t>ESTIMADO — reutilizable: próximos talleres salen mucho más baratos.</t>
       </text>
     </comment>
-    <comment ref="B18" authorId="0" shapeId="0">
+    <comment ref="B31" authorId="0" shapeId="0">
       <text>
-        <t>Copa de vino + pasabocas + café.</t>
+        <t>ESTIMADO — reutilizables.</t>
       </text>
     </comment>
-    <comment ref="B24" authorId="0" shapeId="0">
+    <comment ref="B32" authorId="0" shapeId="0">
       <text>
-        <t>Recomendado para 10–12 personas.</t>
-      </text>
-    </comment>
-    <comment ref="B25" authorId="0" shapeId="0">
-      <text>
-        <t>Imputa un valor aunque sea propio.</t>
-      </text>
-    </comment>
-    <comment ref="A37" authorId="0" shapeId="0">
-      <text>
-        <t>Puedes sobrescribir este precio con el que decidas cobrar; los escenarios de abajo lo usan.</t>
+        <t>Definir el trato con el restaurante (¿pone espacio y comida?).</t>
       </text>
     </comment>
   </commentList>
@@ -554,11 +550,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E48"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
@@ -574,14 +570,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Esmalte + quema · 17 de octubre · 10–12 cupos · refrigerio con vino</t>
+          <t>Esmalte + quema · 17 de octubre · en restaurante · 10–12 cupos · set de 4 pocillos + 4 platos</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Edita solo las celdas AMARILLAS. Los valores son estimados de mercado (Medellín); confírmalos con tus proveedores.</t>
+          <t>Edita solo las celdas AMARILLAS. El refrigerio lo maneja el restaurante (no está en este costo).</t>
         </is>
       </c>
     </row>
@@ -655,374 +651,460 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>COSTOS VARIABLES (por persona)</t>
+          <t>SET DE CERÁMICA (lo que pinta cada persona)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Pieza de cerámica (bisque)</t>
-        </is>
-      </c>
-      <c r="B14" s="7" t="n">
-        <v>20000</v>
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Concepto</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Valor unidad</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Esmaltes y pinturas</t>
-        </is>
-      </c>
-      <c r="B15" s="7" t="n">
-        <v>8000</v>
+          <t>Pocillos</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C15" s="9" t="n">
+        <v>3200</v>
+      </c>
+      <c r="D15" s="10">
+        <f>B15*C15</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Quema por pieza</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="n">
-        <v>12000</v>
+          <t>Platos</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D16" s="10">
+        <f>B16*C16</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>Delantal + empaque</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="n">
-        <v>3000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Refrigerio con vino + pasabocas</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="n">
-        <v>25000</v>
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>Subtotal set por persona</t>
+        </is>
+      </c>
+      <c r="D17" s="12">
+        <f>SUM(D15:D16)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Tarjeta / kit de bienvenida</t>
-        </is>
-      </c>
-      <c r="B19" s="7" t="n">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>OTROS COSTOS VARIABLES (por persona)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Pigmentos (los pone Alado)</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Quema por set</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>Empaque para llevar las piezas</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
         <v>2000</v>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>Subtotal variable por persona</t>
         </is>
       </c>
-      <c r="B20" s="9">
-        <f>SUM(B14:B19)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="B23" s="12">
+        <f>D17+SUM(B20:B22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>COSTOS FIJOS (del evento)</t>
         </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t>Honorarios tallerista (dictado + preparación)</t>
-        </is>
-      </c>
-      <c r="B23" s="7" t="n">
-        <v>400000</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
-        <is>
-          <t>Asistente</t>
-        </is>
-      </c>
-      <c r="B24" s="7" t="n">
-        <v>120000</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Espacio (uso/alquiler, montaje, limpieza)</t>
-        </is>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>200000</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Ambientación (flores, música)</t>
-        </is>
-      </c>
-      <c r="B26" s="7" t="n">
-        <v>80000</v>
+          <t>Lizeth — horas</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Diseño y promoción</t>
-        </is>
-      </c>
-      <c r="B27" s="7" t="n">
-        <v>100000</v>
+          <t>Lizeth — valor hora</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="n">
+        <v>9000</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>Transporte de materiales / piezas a quema</t>
-        </is>
-      </c>
-      <c r="B28" s="7" t="n">
-        <v>60000</v>
+          <t>Lizeth — subtotal</t>
+        </is>
+      </c>
+      <c r="B28" s="10">
+        <f>B26*B27</f>
+        <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="10" t="inlineStr">
-        <is>
-          <t>Subtotal fijos</t>
-        </is>
-      </c>
-      <c r="B29" s="11">
-        <f>SUM(B23:B28)</f>
-        <v/>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Andrés + Alejandro (imputado)</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>Colchón de imprevistos</t>
-        </is>
-      </c>
-      <c r="B30" s="12">
-        <f>B29*B11</f>
-        <v/>
+          <t>Pinceles, esponjas, materiales (compra)</t>
+        </is>
+      </c>
+      <c r="B30" s="9" t="n">
+        <v>200000</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
-        <is>
-          <t>Total fijos (con colchón)</t>
-        </is>
-      </c>
-      <c r="B31" s="9">
-        <f>B29+B30</f>
-        <v/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Delantales (compra)</t>
+        </is>
+      </c>
+      <c r="B31" s="9" t="n">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Espacio (restaurante)</t>
+        </is>
+      </c>
+      <c r="B32" s="9" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="3" t="inlineStr">
-        <is>
-          <t>CÁLCULO DEL PRECIO</t>
-        </is>
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Ambientación (flores, música)</t>
+        </is>
+      </c>
+      <c r="B33" s="9" t="n">
+        <v>50000</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>Costo por persona (al cupo estimado)</t>
-        </is>
-      </c>
-      <c r="B34" s="12">
-        <f>B20+B31/B7</f>
-        <v/>
+          <t>Diseño y promoción</t>
+        </is>
+      </c>
+      <c r="B34" s="9" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t>Transporte de materiales</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
+          <t>Subtotal fijos</t>
+        </is>
+      </c>
+      <c r="B36" s="14">
+        <f>B28+SUM(B29:B35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>Colchón de imprevistos</t>
+        </is>
+      </c>
+      <c r="B37" s="10">
+        <f>B36*B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Total fijos (con colchón)</t>
+        </is>
+      </c>
+      <c r="B38" s="12">
+        <f>B36+B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>CÁLCULO DEL PRECIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>Costo por persona (al cupo estimado)</t>
+        </is>
+      </c>
+      <c r="B41" s="10">
+        <f>B23+B38/B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="4" t="inlineStr">
+        <is>
           <t>Precio por persona (antes de comisión)</t>
         </is>
       </c>
-      <c r="B35" s="12">
-        <f>B34/(1-B9)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
+      <c r="B42" s="10">
+        <f>B41/(1-B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
         <is>
           <t>Precio por persona (cubriendo comisión)</t>
         </is>
       </c>
-      <c r="B36" s="12">
-        <f>B35/(1-B10)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="B43" s="10">
+        <f>B42/(1-B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>PRECIO SUGERIDO POR CUPO (redondeado)</t>
         </is>
       </c>
-      <c r="B37" s="14">
-        <f>ROUND(B36/5000,0)*5000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="B44" s="16">
+        <f>ROUND(B43/5000,0)*5000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>PUNTO DE EQUILIBRIO Y ESCENARIOS</t>
         </is>
       </c>
     </row>
-    <row r="40">
-      <c r="A40" s="4" t="inlineStr">
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
         <is>
           <t>Precio de venta usado</t>
         </is>
       </c>
-      <c r="B40" s="12">
-        <f>B37</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="10" t="inlineStr">
+      <c r="B47" s="10">
+        <f>B44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="13" t="inlineStr">
         <is>
           <t>Punto de equilibrio (nº personas)</t>
         </is>
       </c>
-      <c r="B41" s="15">
-        <f>ROUNDUP(B31/(B40*(1-B10)-B20),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="B48" s="17">
+        <f>ROUNDUP(B38/(B47*(1-B10)-B23),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="18" t="inlineStr">
         <is>
           <t>Escenario</t>
         </is>
       </c>
-      <c r="B43" s="16" t="inlineStr">
+      <c r="B50" s="18" t="inlineStr">
         <is>
           <t>Personas</t>
         </is>
       </c>
-      <c r="C43" s="16" t="inlineStr">
+      <c r="C50" s="18" t="inlineStr">
         <is>
           <t>Ingresos</t>
         </is>
       </c>
-      <c r="D43" s="16" t="inlineStr">
+      <c r="D50" s="18" t="inlineStr">
         <is>
           <t>Costos totales</t>
         </is>
       </c>
-      <c r="E43" s="16" t="inlineStr">
+      <c r="E50" s="18" t="inlineStr">
         <is>
           <t>Ganancia</t>
         </is>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="17" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="19" t="inlineStr">
         <is>
           <t>Mínimo</t>
         </is>
       </c>
-      <c r="B44" s="18">
+      <c r="B51" s="20">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C44" s="12">
-        <f>$B$40*B44</f>
-        <v/>
-      </c>
-      <c r="D44" s="12">
-        <f>$B$31+$B$20*B44+$B$10*C44</f>
-        <v/>
-      </c>
-      <c r="E44" s="11">
-        <f>C44-D44</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="17" t="inlineStr">
+      <c r="C51" s="10">
+        <f>$B$47*B51</f>
+        <v/>
+      </c>
+      <c r="D51" s="10">
+        <f>$B$38+$B$23*B51+$B$10*C51</f>
+        <v/>
+      </c>
+      <c r="E51" s="14">
+        <f>C51-D51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="19" t="inlineStr">
         <is>
           <t>Estimado</t>
         </is>
       </c>
-      <c r="B45" s="18">
+      <c r="B52" s="20">
         <f>B7</f>
         <v/>
       </c>
-      <c r="C45" s="12">
-        <f>$B$40*B45</f>
-        <v/>
-      </c>
-      <c r="D45" s="12">
-        <f>$B$31+$B$20*B45+$B$10*C45</f>
-        <v/>
-      </c>
-      <c r="E45" s="11">
-        <f>C45-D45</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="17" t="inlineStr">
+      <c r="C52" s="10">
+        <f>$B$47*B52</f>
+        <v/>
+      </c>
+      <c r="D52" s="10">
+        <f>$B$38+$B$23*B52+$B$10*C52</f>
+        <v/>
+      </c>
+      <c r="E52" s="14">
+        <f>C52-D52</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="19" t="inlineStr">
         <is>
           <t>Máximo</t>
         </is>
       </c>
-      <c r="B46" s="18">
+      <c r="B53" s="20">
         <f>B8</f>
         <v/>
       </c>
-      <c r="C46" s="12">
-        <f>$B$40*B46</f>
-        <v/>
-      </c>
-      <c r="D46" s="12">
-        <f>$B$31+$B$20*B46+$B$10*C46</f>
-        <v/>
-      </c>
-      <c r="E46" s="11">
-        <f>C46-D46</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>Nota: estimados de mercado de Medellín para taller de cerámica con esmalte+quema y refrigerio. Ajusta cada celda amarilla con tus cifras reales.</t>
+      <c r="C53" s="10">
+        <f>$B$47*B53</f>
+        <v/>
+      </c>
+      <c r="D53" s="10">
+        <f>$B$38+$B$23*B53+$B$10*C53</f>
+        <v/>
+      </c>
+      <c r="E53" s="14">
+        <f>C53-D53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Nota: pinceles, esponjas, materiales y delantales son reutilizables → los próximos talleres cuestan mucho menos. Pigmentos y quema son estimados (confirmar).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A39:E39"/>
-    <mergeCell ref="A48:E48"/>
+  <mergeCells count="10">
+    <mergeCell ref="A55:E55"/>
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A33:E33"/>
+    <mergeCell ref="A25:E25"/>
+    <mergeCell ref="A19:E19"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A46:E46"/>
     <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Workshop Excel: add cupo price, margin, profit, break-even and scenarios
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
@@ -16,8 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -105,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -113,11 +114,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -192,6 +207,86 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Alado</author>
+  </authors>
+  <commentList>
+    <comment ref="B8" authorId="0" shapeId="0">
+      <text>
+        <t>Ganancia dividida entre lo que cobras. 40% = de cada $100 cobrados, $40 son ganancia.</t>
+      </text>
+    </comment>
+    <comment ref="B10" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Pon 0% si no quieres colchón.</t>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara: taller amigo.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO.</t>
+      </text>
+    </comment>
+    <comment ref="B18" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B19" authorId="0" shapeId="0">
+      <text>
+        <t>Dato de Sara.</t>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Son reutilizables: en el próximo taller cuestan menos.</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO. Reutilizables.</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>ESTIMADO.</t>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0">
+      <text>
+        <t>Invitación, cómo participar, historias y recap. Pon $0 si no se carga al taller.</t>
+      </text>
+    </comment>
+    <comment ref="B24" authorId="0" shapeId="0">
+      <text>
+        <t>Lo que se acuerde con el restaurante. Pon $0 si no hay pago.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -483,302 +578,731 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B33"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Taller de pintura en cerámica — Cotización</t>
+          <t>Taller de pintura en cerámica · precio del cupo, margen y ganancia</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>17 de octubre · en restaurante (ellos ponen lugar, aperitivos y vino)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>✏️  EDITA ESTO (celdas amarillas)</t>
+          <t>17 de octubre · en restaurante (ellos ponen lugar, aperitivos y vino) · esmalte + quema</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Edita solo las celdas AMARILLAS. Todo lo demás se calcula solo.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>Nº de personas</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n">
-        <v>11</v>
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>EDITA ESTO</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Pocillos por persona (cantidad)</t>
+          <t>Nº de personas</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Precio de 1 pocillo</t>
+          <t>Precio del cupo (lo que cobras)</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>3200</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Platos por persona (cantidad)</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n">
-        <v>4</v>
+          <t>Margen de ganancia que quieres (sobre ventas)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Precio de 1 plato</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n">
-        <v>2200</v>
+          <t>Comisión de pago online (0% si es transferencia)</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Pigmentos (por persona)</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="n">
-        <v>6000</v>
+          <t>Imprevistos (% de los costos)</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Quema (por pieza)</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="n">
-        <v>3000</v>
+          <t>Pocillos por persona (cantidad)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Empaque (por persona)</t>
+          <t>Precio de 1 pocillo</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>2000</v>
+        <v>3200</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Lizeth — horas</t>
+          <t>Platos por persona (cantidad)</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>Lizeth — valor por hora</t>
+          <t>Precio de 1 plato</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>9000</v>
+        <v>2200</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Pinceles, esponjas y materiales (total)</t>
+          <t>Pigmentos (por persona)</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>200000</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Delantales (total)</t>
+          <t>Quema (por pieza)</t>
         </is>
       </c>
       <c r="B16" s="6" t="n">
-        <v>120000</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Otros fijos: transporte, flores, promo (total)</t>
+          <t>Empaque (por persona)</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>190000</v>
+        <v>2000</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>PRECIO por persona (lo que cobras)</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="n">
-        <v>200000</v>
+          <t>Lizeth · horas</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Lo que quieres ganar (mínimo)</t>
+          <t>Lizeth · valor por hora</t>
         </is>
       </c>
       <c r="B19" s="6" t="n">
-        <v>600000</v>
+        <v>9000</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Pinceles, esponjas y materiales (total)</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>200000</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>📊  RESULTADO (se calcula solo)</t>
-        </is>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>Delantales (total)</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>120000</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Piezas por persona</t>
-        </is>
-      </c>
-      <c r="B22" s="7">
-        <f>B6+B8</f>
-        <v/>
+          <t>Otros fijos: transporte, flores, promoción (total)</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>190000</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Costo variable por persona</t>
-        </is>
-      </c>
-      <c r="B23" s="8">
-        <f>(B6*B7)+(B8*B9)+B10+((B6+B8)*B11)+B12</f>
-        <v/>
+          <t>Contenido del taller (4 piezas de Sara)</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>690000</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Costo fijo total</t>
-        </is>
-      </c>
-      <c r="B24" s="8">
-        <f>(B13*B14)+B15+B16+B17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Costo total del taller</t>
-        </is>
-      </c>
-      <c r="B25" s="8">
-        <f>B24+B23*B5</f>
-        <v/>
+          <t>Pago al restaurante (total)</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>Ingresos (precio × personas)</t>
-        </is>
-      </c>
-      <c r="B26" s="8">
-        <f>B18*B5</f>
-        <v/>
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>RESULTADO</t>
+        </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="9" t="inlineStr">
-        <is>
-          <t>Ganancia (antes de pagar al restaurante)</t>
-        </is>
-      </c>
-      <c r="B27" s="10">
-        <f>B26-B25</f>
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>Piezas por persona</t>
+        </is>
+      </c>
+      <c r="B27" s="8">
+        <f>B11+B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Costo variable por persona (cerámica, pigmentos, quema, empaque)</t>
+        </is>
+      </c>
+      <c r="B28" s="9">
+        <f>B11*B12+B13*B14+B15+(B11+B13)*B16+B17</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>👉 PUEDES PAGARLE AL RESTAURANTE (máx, total)</t>
-        </is>
-      </c>
-      <c r="B29" s="6">
-        <f>B27-B19</f>
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Costos fijos (Lizeth, materiales, delantales, otros y contenido)</t>
+        </is>
+      </c>
+      <c r="B29" s="9">
+        <f>B18*B19+B20+B21+B22+B23</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">      … por persona</t>
-        </is>
-      </c>
-      <c r="B30" s="11">
-        <f>B29/B5</f>
+          <t>Costos base (fijos + variables × personas)</t>
+        </is>
+      </c>
+      <c r="B30" s="9">
+        <f>B29+B28*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Imprevistos</t>
+        </is>
+      </c>
+      <c r="B31" s="9">
+        <f>B30*B10</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>Cambia el PRECIO (fila 18) o lo que quieres ganar (fila 19) y mira cuánto puedes pagarle al restaurante.</t>
-        </is>
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>Pago al restaurante</t>
+        </is>
+      </c>
+      <c r="B32" s="9">
+        <f>B24</f>
+        <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>Nota: pinceles, esponjas y delantales son reutilizables → próximos talleres cuestan menos.</t>
+      <c r="A33" s="10" t="inlineStr">
+        <is>
+          <t>COSTO TOTAL del taller</t>
+        </is>
+      </c>
+      <c r="B33" s="11">
+        <f>B30+B31+B32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>Costo por persona</t>
+        </is>
+      </c>
+      <c r="B34" s="9">
+        <f>B33/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos por cupos (precio × personas)</t>
+        </is>
+      </c>
+      <c r="B35" s="9">
+        <f>B7*B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t>Comisión de pago online</t>
+        </is>
+      </c>
+      <c r="B36" s="9">
+        <f>B35*B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="10" t="inlineStr">
+        <is>
+          <t>GANANCIA</t>
+        </is>
+      </c>
+      <c r="B37" s="11">
+        <f>B35-B36-B33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="10" t="inlineStr">
+        <is>
+          <t>MARGEN real (ganancia ÷ ingresos)</t>
+        </is>
+      </c>
+      <c r="B38" s="12">
+        <f>IF(B35&gt;0,B37/B35,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>Ganancia por persona</t>
+        </is>
+      </c>
+      <c r="B39" s="9">
+        <f>B37/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>¿Cumple el margen que quieres?</t>
+        </is>
+      </c>
+      <c r="B40" s="13">
+        <f>IF(B38&gt;=B8,"Sí, cumple","No: está por debajo")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>CUÁNTO DEBE VALER EL CUPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>Precio mínimo (no pierdes ni ganas)</t>
+        </is>
+      </c>
+      <c r="B43" s="9">
+        <f>B33/(B6*(1-B9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="10" t="inlineStr">
+        <is>
+          <t>PRECIO RECOMENDADO para tu margen (redondeado a $5.000)</t>
+        </is>
+      </c>
+      <c r="B44" s="14">
+        <f>IF(1-B9-B8&lt;=0,"Revisa el margen",ROUNDUP(B33/(B6*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>Diferencia con el precio que cobras hoy</t>
+        </is>
+      </c>
+      <c r="B45" s="9">
+        <f>IF(ISNUMBER(B44),B44-B7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="4" t="inlineStr">
+        <is>
+          <t>Punto de equilibrio (personas para no perder)</t>
+        </is>
+      </c>
+      <c r="B46" s="8">
+        <f>IF(B7*(1-B9)-B28*(1+B10)&gt;0,ROUNDUP((B29*(1+B10)+B24)/(B7*(1-B9)-B28*(1+B10)),0),"No alcanza con este precio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>Máximo que puedes pagar al restaurante y mantener tu margen</t>
+        </is>
+      </c>
+      <c r="B47" s="9">
+        <f>B35*(1-B9-B8)-(B30+B31)</f>
+        <v/>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>(negativo = el precio no alcanza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>PRECIO DEL CUPO SEGÚN EL MARGEN QUE QUIERAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>Precio del cupo</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Ganancia total</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B51" s="9">
+        <f>IF(1-$B$9-A51&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A51))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C51" s="9">
+        <f>IF(ISNUMBER(B51),B51*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B52" s="9">
+        <f>IF(1-$B$9-A52&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A52))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C52" s="9">
+        <f>IF(ISNUMBER(B52),B52*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B53" s="9">
+        <f>IF(1-$B$9-A53&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A53))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C53" s="9">
+        <f>IF(ISNUMBER(B53),B53*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B54" s="9">
+        <f>IF(1-$B$9-A54&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A54))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C54" s="9">
+        <f>IF(ISNUMBER(B54),B54*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="15" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="B57" s="15" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="C57" s="15" t="inlineStr">
+        <is>
+          <t>Costo total</t>
+        </is>
+      </c>
+      <c r="D57" s="15" t="inlineStr">
+        <is>
+          <t>Ganancia</t>
+        </is>
+      </c>
+      <c r="E57" s="15" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+      <c r="F57" s="15" t="inlineStr">
+        <is>
+          <t>Precio para tu margen</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="n">
+        <v>6</v>
+      </c>
+      <c r="B58" s="9">
+        <f>$B$7*A58</f>
+        <v/>
+      </c>
+      <c r="C58" s="9">
+        <f>($B$29+$B$28*A58)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D58" s="18">
+        <f>B58*(1-$B$9)-C58</f>
+        <v/>
+      </c>
+      <c r="E58" s="19">
+        <f>IF(B58&gt;0,D58/B58,0)</f>
+        <v/>
+      </c>
+      <c r="F58" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C58/(A58*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B59" s="9">
+        <f>$B$7*A59</f>
+        <v/>
+      </c>
+      <c r="C59" s="9">
+        <f>($B$29+$B$28*A59)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D59" s="18">
+        <f>B59*(1-$B$9)-C59</f>
+        <v/>
+      </c>
+      <c r="E59" s="19">
+        <f>IF(B59&gt;0,D59/B59,0)</f>
+        <v/>
+      </c>
+      <c r="F59" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C59/(A59*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="B60" s="9">
+        <f>$B$7*A60</f>
+        <v/>
+      </c>
+      <c r="C60" s="9">
+        <f>($B$29+$B$28*A60)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D60" s="18">
+        <f>B60*(1-$B$9)-C60</f>
+        <v/>
+      </c>
+      <c r="E60" s="19">
+        <f>IF(B60&gt;0,D60/B60,0)</f>
+        <v/>
+      </c>
+      <c r="F60" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C60/(A60*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="B61" s="9">
+        <f>$B$7*A61</f>
+        <v/>
+      </c>
+      <c r="C61" s="9">
+        <f>($B$29+$B$28*A61)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D61" s="18">
+        <f>B61*(1-$B$9)-C61</f>
+        <v/>
+      </c>
+      <c r="E61" s="19">
+        <f>IF(B61&gt;0,D61/B61,0)</f>
+        <v/>
+      </c>
+      <c r="F61" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C61/(A61*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="B62" s="9">
+        <f>$B$7*A62</f>
+        <v/>
+      </c>
+      <c r="C62" s="9">
+        <f>($B$29+$B$28*A62)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D62" s="18">
+        <f>B62*(1-$B$9)-C62</f>
+        <v/>
+      </c>
+      <c r="E62" s="19">
+        <f>IF(B62&gt;0,D62/B62,0)</f>
+        <v/>
+      </c>
+      <c r="F62" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C62/(A62*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Nota: pinceles, esponjas y delantales se compran una vez; en los próximos talleres el costo fijo baja. Los datos marcados ESTIMADO no son cotizaciones reales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>El restaurante pone lugar, aperitivos y vino; por eso esos costos no aparecen aquí.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="A33:B33"/>
-    <mergeCell ref="A32:B32"/>
-    <mergeCell ref="A1:B1"/>
+  <mergeCells count="10">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A49:F49"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A64:F64"/>
+    <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Workshop Excel: dedicated break-even section and per-scenario coverage
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
@@ -106,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -122,6 +122,7 @@
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -578,15 +579,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="58" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1011,296 +1013,373 @@
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Punto de equilibrio (personas para no perder)</t>
-        </is>
-      </c>
-      <c r="B46" s="8">
+          <t>Máximo que puedes pagar al restaurante y mantener tu margen</t>
+        </is>
+      </c>
+      <c r="B46" s="9">
+        <f>B35*(1-B9-B8)-(B30+B31)</f>
+        <v/>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>(negativo = el precio no alcanza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>PUNTO DE EQUILIBRIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="10" t="inlineStr">
+        <is>
+          <t>Personas necesarias para no perder</t>
+        </is>
+      </c>
+      <c r="B49" s="15">
         <f>IF(B7*(1-B9)-B28*(1+B10)&gt;0,ROUNDUP((B29*(1+B10)+B24)/(B7*(1-B9)-B28*(1+B10)),0),"No alcanza con este precio")</f>
         <v/>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="4" t="inlineStr">
-        <is>
-          <t>Máximo que puedes pagar al restaurante y mantener tu margen</t>
-        </is>
-      </c>
-      <c r="B47" s="9">
-        <f>B35*(1-B9-B8)-(B30+B31)</f>
-        <v/>
-      </c>
-      <c r="C47" s="2" t="inlineStr">
-        <is>
-          <t>(negativo = el precio no alcanza)</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="3" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos necesarios para no perder</t>
+        </is>
+      </c>
+      <c r="B50" s="9">
+        <f>IF(ISNUMBER(B49),B49*B7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>Aporte de cada cupo a los costos fijos (precio menos su costo variable)</t>
+        </is>
+      </c>
+      <c r="B51" s="9">
+        <f>B7*(1-B9)-B28*(1+B10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="4" t="inlineStr">
+        <is>
+          <t>Personas por encima (+) o por debajo (−) del equilibrio</t>
+        </is>
+      </c>
+      <c r="B52" s="8">
+        <f>IF(ISNUMBER(B49),B6-B49,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>¿Con tu número de personas cubres costos?</t>
+        </is>
+      </c>
+      <c r="B53" s="13">
+        <f>IF(ISNUMBER(B49),IF(B6&gt;=B49,"Sí, cubres costos","No, pierdes dinero"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>PRECIO DEL CUPO SEGÚN EL MARGEN QUE QUIERAS</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="15" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="16" t="inlineStr">
         <is>
           <t>Margen</t>
         </is>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B56" s="16" t="inlineStr">
         <is>
           <t>Precio del cupo</t>
         </is>
       </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="C56" s="16" t="inlineStr">
         <is>
           <t>Ganancia total</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="16" t="n">
+    <row r="57">
+      <c r="A57" s="17" t="n">
         <v>0.2</v>
       </c>
-      <c r="B51" s="9">
-        <f>IF(1-$B$9-A51&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A51))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C51" s="9">
-        <f>IF(ISNUMBER(B51),B51*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B52" s="9">
-        <f>IF(1-$B$9-A52&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A52))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C52" s="9">
-        <f>IF(ISNUMBER(B52),B52*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="B53" s="9">
-        <f>IF(1-$B$9-A53&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A53))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C53" s="9">
-        <f>IF(ISNUMBER(B53),B53*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B54" s="9">
-        <f>IF(1-$B$9-A54&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A54))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C54" s="9">
-        <f>IF(ISNUMBER(B54),B54*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
-        <is>
-          <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="15" t="inlineStr">
-        <is>
-          <t>Personas</t>
-        </is>
-      </c>
-      <c r="B57" s="15" t="inlineStr">
-        <is>
-          <t>Ingresos</t>
-        </is>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
-        <is>
-          <t>Costo total</t>
-        </is>
-      </c>
-      <c r="D57" s="15" t="inlineStr">
-        <is>
-          <t>Ganancia</t>
-        </is>
-      </c>
-      <c r="E57" s="15" t="inlineStr">
-        <is>
-          <t>Margen</t>
-        </is>
-      </c>
-      <c r="F57" s="15" t="inlineStr">
-        <is>
-          <t>Precio para tu margen</t>
-        </is>
+      <c r="B57" s="9">
+        <f>IF(1-$B$9-A57&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A57))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C57" s="9">
+        <f>IF(ISNUMBER(B57),B57*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="17" t="n">
-        <v>6</v>
+        <v>0.3</v>
       </c>
       <c r="B58" s="9">
-        <f>$B$7*A58</f>
+        <f>IF(1-$B$9-A58&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A58))/5000,0)*5000)</f>
         <v/>
       </c>
       <c r="C58" s="9">
-        <f>($B$29+$B$28*A58)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D58" s="18">
-        <f>B58*(1-$B$9)-C58</f>
-        <v/>
-      </c>
-      <c r="E58" s="19">
-        <f>IF(B58&gt;0,D58/B58,0)</f>
-        <v/>
-      </c>
-      <c r="F58" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C58/(A58*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <f>IF(ISNUMBER(B58),B58*$B$6*(1-$B$9)-$B$33,"")</f>
         <v/>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="17" t="n">
-        <v>8</v>
+        <v>0.4</v>
       </c>
       <c r="B59" s="9">
-        <f>$B$7*A59</f>
+        <f>IF(1-$B$9-A59&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A59))/5000,0)*5000)</f>
         <v/>
       </c>
       <c r="C59" s="9">
-        <f>($B$29+$B$28*A59)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D59" s="18">
-        <f>B59*(1-$B$9)-C59</f>
-        <v/>
-      </c>
-      <c r="E59" s="19">
-        <f>IF(B59&gt;0,D59/B59,0)</f>
-        <v/>
-      </c>
-      <c r="F59" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C59/(A59*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <f>IF(ISNUMBER(B59),B59*$B$6*(1-$B$9)-$B$33,"")</f>
         <v/>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B60" s="9">
+        <f>IF(1-$B$9-A60&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A60))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C60" s="9">
+        <f>IF(ISNUMBER(B60),B60*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="16" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="C63" s="16" t="inlineStr">
+        <is>
+          <t>Costo total</t>
+        </is>
+      </c>
+      <c r="D63" s="16" t="inlineStr">
+        <is>
+          <t>Ganancia</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+      <c r="F63" s="16" t="inlineStr">
+        <is>
+          <t>Precio para tu margen</t>
+        </is>
+      </c>
+      <c r="G63" s="16" t="inlineStr">
+        <is>
+          <t>¿Cubre costos?</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B64" s="9">
+        <f>$B$7*A64</f>
+        <v/>
+      </c>
+      <c r="C64" s="9">
+        <f>($B$29+$B$28*A64)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D64" s="19">
+        <f>B64*(1-$B$9)-C64</f>
+        <v/>
+      </c>
+      <c r="E64" s="20">
+        <f>IF(B64&gt;0,D64/B64,0)</f>
+        <v/>
+      </c>
+      <c r="F64" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C64/(A64*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G64" s="13">
+        <f>IF(D64&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="B65" s="9">
+        <f>$B$7*A65</f>
+        <v/>
+      </c>
+      <c r="C65" s="9">
+        <f>($B$29+$B$28*A65)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D65" s="19">
+        <f>B65*(1-$B$9)-C65</f>
+        <v/>
+      </c>
+      <c r="E65" s="20">
+        <f>IF(B65&gt;0,D65/B65,0)</f>
+        <v/>
+      </c>
+      <c r="F65" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C65/(A65*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G65" s="13">
+        <f>IF(D65&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="B60" s="9">
-        <f>$B$7*A60</f>
-        <v/>
-      </c>
-      <c r="C60" s="9">
-        <f>($B$29+$B$28*A60)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D60" s="18">
-        <f>B60*(1-$B$9)-C60</f>
-        <v/>
-      </c>
-      <c r="E60" s="19">
-        <f>IF(B60&gt;0,D60/B60,0)</f>
-        <v/>
-      </c>
-      <c r="F60" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C60/(A60*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="17" t="n">
+      <c r="B66" s="9">
+        <f>$B$7*A66</f>
+        <v/>
+      </c>
+      <c r="C66" s="9">
+        <f>($B$29+$B$28*A66)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D66" s="19">
+        <f>B66*(1-$B$9)-C66</f>
+        <v/>
+      </c>
+      <c r="E66" s="20">
+        <f>IF(B66&gt;0,D66/B66,0)</f>
+        <v/>
+      </c>
+      <c r="F66" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C66/(A66*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G66" s="13">
+        <f>IF(D66&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="18" t="n">
         <v>11</v>
       </c>
-      <c r="B61" s="9">
-        <f>$B$7*A61</f>
-        <v/>
-      </c>
-      <c r="C61" s="9">
-        <f>($B$29+$B$28*A61)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D61" s="18">
-        <f>B61*(1-$B$9)-C61</f>
-        <v/>
-      </c>
-      <c r="E61" s="19">
-        <f>IF(B61&gt;0,D61/B61,0)</f>
-        <v/>
-      </c>
-      <c r="F61" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C61/(A61*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="17" t="n">
+      <c r="B67" s="9">
+        <f>$B$7*A67</f>
+        <v/>
+      </c>
+      <c r="C67" s="9">
+        <f>($B$29+$B$28*A67)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D67" s="19">
+        <f>B67*(1-$B$9)-C67</f>
+        <v/>
+      </c>
+      <c r="E67" s="20">
+        <f>IF(B67&gt;0,D67/B67,0)</f>
+        <v/>
+      </c>
+      <c r="F67" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C67/(A67*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G67" s="13">
+        <f>IF(D67&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="B62" s="9">
-        <f>$B$7*A62</f>
-        <v/>
-      </c>
-      <c r="C62" s="9">
-        <f>($B$29+$B$28*A62)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D62" s="18">
-        <f>B62*(1-$B$9)-C62</f>
-        <v/>
-      </c>
-      <c r="E62" s="19">
-        <f>IF(B62&gt;0,D62/B62,0)</f>
-        <v/>
-      </c>
-      <c r="F62" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C62/(A62*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="inlineStr">
+      <c r="B68" s="9">
+        <f>$B$7*A68</f>
+        <v/>
+      </c>
+      <c r="C68" s="9">
+        <f>($B$29+$B$28*A68)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D68" s="19">
+        <f>B68*(1-$B$9)-C68</f>
+        <v/>
+      </c>
+      <c r="E68" s="20">
+        <f>IF(B68&gt;0,D68/B68,0)</f>
+        <v/>
+      </c>
+      <c r="F68" s="9">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C68/(A68*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G68" s="13">
+        <f>IF(D68&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
         <is>
           <t>Nota: pinceles, esponjas y delantales se compran una vez; en los próximos talleres el costo fijo baja. Los datos marcados ESTIMADO no son cotizaciones reales.</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="2" t="inlineStr">
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
         <is>
           <t>El restaurante pone lugar, aperitivos y vino; por eso esos costos no aparecen aquí.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A49:F49"/>
-    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A70:G70"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A5:F5"/>
-    <mergeCell ref="A26:F26"/>
-    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A55:G55"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A62:G62"/>
+    <mergeCell ref="A42:G42"/>
     <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A64:F64"/>
-    <mergeCell ref="A65:F65"/>
+    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>

</xml_diff>

<commit_message>
Workshop Excel: restaurant payment section with suggested amount and editable agreed payment
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FV7y6XEE3x9ogCMyfe3pnd
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
@@ -115,12 +115,13 @@
     <xf numFmtId="1" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -133,7 +134,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -281,9 +281,14 @@
         <t>Invitación, cómo participar, historias y recap. Pon $0 si no se carga al taller.</t>
       </text>
     </comment>
-    <comment ref="B24" authorId="0" shapeId="0">
+    <comment ref="B44" authorId="0" shapeId="0">
       <text>
-        <t>Lo que se acuerde con el restaurante. Pon $0 si no hay pago.</t>
+        <t>Es una propuesta de partida. Súbelo o bájalo según lo que negocies.</t>
+      </text>
+    </comment>
+    <comment ref="B47" authorId="0" shapeId="0">
+      <text>
+        <t>Escribe el valor que acuerdes con el restaurante. La ganancia de abajo se recalcula sola.</t>
       </text>
     </comment>
   </commentList>
@@ -579,10 +584,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="64" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
@@ -802,11 +807,12 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Pago al restaurante (total)</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="n">
-        <v>0</v>
+          <t>Pago al restaurante (total) · se escribe en la sección «Pago al restaurante»</t>
+        </is>
+      </c>
+      <c r="B24" s="8">
+        <f>B47</f>
+        <v/>
       </c>
     </row>
     <row r="26">
@@ -822,7 +828,7 @@
           <t>Piezas por persona</t>
         </is>
       </c>
-      <c r="B27" s="8">
+      <c r="B27" s="9">
         <f>B11+B13</f>
         <v/>
       </c>
@@ -833,7 +839,7 @@
           <t>Costo variable por persona (cerámica, pigmentos, quema, empaque)</t>
         </is>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="8">
         <f>B11*B12+B13*B14+B15+(B11+B13)*B16+B17</f>
         <v/>
       </c>
@@ -844,7 +850,7 @@
           <t>Costos fijos (Lizeth, materiales, delantales, otros y contenido)</t>
         </is>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="8">
         <f>B18*B19+B20+B21+B22+B23</f>
         <v/>
       </c>
@@ -855,7 +861,7 @@
           <t>Costos base (fijos + variables × personas)</t>
         </is>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="8">
         <f>B29+B28*B6</f>
         <v/>
       </c>
@@ -866,7 +872,7 @@
           <t>Imprevistos</t>
         </is>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="8">
         <f>B30*B10</f>
         <v/>
       </c>
@@ -877,7 +883,7 @@
           <t>Pago al restaurante</t>
         </is>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="8">
         <f>B24</f>
         <v/>
       </c>
@@ -899,7 +905,7 @@
           <t>Costo por persona</t>
         </is>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="8">
         <f>B33/B6</f>
         <v/>
       </c>
@@ -910,7 +916,7 @@
           <t>Ingresos por cupos (precio × personas)</t>
         </is>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="8">
         <f>B7*B6</f>
         <v/>
       </c>
@@ -921,7 +927,7 @@
           <t>Comisión de pago online</t>
         </is>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="8">
         <f>B35*B9</f>
         <v/>
       </c>
@@ -929,7 +935,7 @@
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
-          <t>GANANCIA</t>
+          <t>GANANCIA (después de pagarle al restaurante)</t>
         </is>
       </c>
       <c r="B37" s="11">
@@ -954,7 +960,7 @@
           <t>Ganancia por persona</t>
         </is>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="8">
         <f>B37/B6</f>
         <v/>
       </c>
@@ -973,412 +979,517 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>CUÁNTO DEBE VALER EL CUPO</t>
+          <t>PAGO AL RESTAURANTE</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>Precio mínimo (no pierdes ni ganas)</t>
-        </is>
-      </c>
-      <c r="B43" s="9">
-        <f>B33/(B6*(1-B9))</f>
+          <t>Ganancia antes de pagarle al restaurante</t>
+        </is>
+      </c>
+      <c r="B43" s="8">
+        <f>B35-B36-(B30+B31)</f>
         <v/>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>PRECIO RECOMENDADO para tu margen (redondeado a $5.000)</t>
-        </is>
-      </c>
-      <c r="B44" s="14">
-        <f>IF(1-B9-B8&lt;=0,"Revisa el margen",ROUNDUP(B33/(B6*(1-B9-B8))/5000,0)*5000)</f>
-        <v/>
+      <c r="A44" s="4" t="inlineStr">
+        <is>
+          <t>% de esa ganancia que le ofreces al restaurante</t>
+        </is>
+      </c>
+      <c r="B44" s="7" t="n">
+        <v>0.3</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
-        <is>
-          <t>Diferencia con el precio que cobras hoy</t>
-        </is>
-      </c>
-      <c r="B45" s="9">
-        <f>IF(ISNUMBER(B44),B44-B7,"")</f>
+      <c r="A45" s="10" t="inlineStr">
+        <is>
+          <t>PAGO SUGERIDO al restaurante (redondeado a $5.000)</t>
+        </is>
+      </c>
+      <c r="B45" s="11">
+        <f>MAX(0,ROUNDDOWN(B43*B44/5000,0)*5000)</f>
         <v/>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>Máximo que puedes pagar al restaurante y mantener tu margen</t>
-        </is>
-      </c>
-      <c r="B46" s="9">
-        <f>B35*(1-B9-B8)-(B30+B31)</f>
-        <v/>
-      </c>
-      <c r="C46" s="2" t="inlineStr">
-        <is>
-          <t>(negativo = el precio no alcanza)</t>
-        </is>
+          <t>…por persona</t>
+        </is>
+      </c>
+      <c r="B46" s="8">
+        <f>B45/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>LO QUE ACUERDAS PAGAR (escribe aquí)</t>
+        </is>
+      </c>
+      <c r="B47" s="6" t="n">
+        <v>80000</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
-        <is>
-          <t>PUNTO DE EQUILIBRIO</t>
-        </is>
+      <c r="A48" s="10" t="inlineStr">
+        <is>
+          <t>TU GANANCIA después de pagarle</t>
+        </is>
+      </c>
+      <c r="B48" s="11">
+        <f>B43-B47</f>
+        <v/>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="10" t="inlineStr">
-        <is>
-          <t>Personas necesarias para no perder</t>
-        </is>
-      </c>
-      <c r="B49" s="15">
-        <f>IF(B7*(1-B9)-B28*(1+B10)&gt;0,ROUNDUP((B29*(1+B10)+B24)/(B7*(1-B9)-B28*(1+B10)),0),"No alcanza con este precio")</f>
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>Tu margen después de pagarle</t>
+        </is>
+      </c>
+      <c r="B49" s="14">
+        <f>IF(B35&gt;0,B48/B35,0)</f>
         <v/>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>Ingresos necesarios para no perder</t>
-        </is>
-      </c>
-      <c r="B50" s="9">
-        <f>IF(ISNUMBER(B49),B49*B7,"")</f>
+          <t>Máximo que puedes pagar sin perder dinero</t>
+        </is>
+      </c>
+      <c r="B50" s="8">
+        <f>MAX(0,B43)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
+          <t>Aviso</t>
+        </is>
+      </c>
+      <c r="B51" s="13">
+        <f>IF(B47&gt;B43,"Cuidado: con ese pago pierdes dinero",IF(B49&lt;B8,"Ganas, pero por debajo de tu margen","Cumples tu margen"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>CUÁNTO DEBE VALER EL CUPO</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="4" t="inlineStr">
+        <is>
+          <t>Precio mínimo (no pierdes ni ganas)</t>
+        </is>
+      </c>
+      <c r="B54" s="8">
+        <f>B33/(B6*(1-B9))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="10" t="inlineStr">
+        <is>
+          <t>PRECIO RECOMENDADO para tu margen (redondeado a $5.000)</t>
+        </is>
+      </c>
+      <c r="B55" s="15">
+        <f>IF(1-B9-B8&lt;=0,"Revisa el margen",ROUNDUP(B33/(B6*(1-B9-B8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="4" t="inlineStr">
+        <is>
+          <t>Diferencia con el precio que cobras hoy</t>
+        </is>
+      </c>
+      <c r="B56" s="8">
+        <f>IF(ISNUMBER(B55),B55-B7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>Máximo que puedes pagar al restaurante y mantener tu margen</t>
+        </is>
+      </c>
+      <c r="B57" s="8">
+        <f>B35*(1-B9-B8)-(B30+B31)</f>
+        <v/>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>(negativo = el precio no alcanza)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
+          <t>PUNTO DE EQUILIBRIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="10" t="inlineStr">
+        <is>
+          <t>Personas necesarias para no perder</t>
+        </is>
+      </c>
+      <c r="B60" s="16">
+        <f>IF(B7*(1-B9)-B28*(1+B10)&gt;0,ROUNDUP((B29*(1+B10)+B24)/(B7*(1-B9)-B28*(1+B10)),0),"No alcanza con este precio")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>Ingresos necesarios para no perder</t>
+        </is>
+      </c>
+      <c r="B61" s="8">
+        <f>IF(ISNUMBER(B60),B60*B7,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
           <t>Aporte de cada cupo a los costos fijos (precio menos su costo variable)</t>
         </is>
       </c>
-      <c r="B51" s="9">
+      <c r="B62" s="8">
         <f>B7*(1-B9)-B28*(1+B10)</f>
         <v/>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="4" t="inlineStr">
         <is>
           <t>Personas por encima (+) o por debajo (−) del equilibrio</t>
         </is>
       </c>
-      <c r="B52" s="8">
-        <f>IF(ISNUMBER(B49),B6-B49,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="4" t="inlineStr">
+      <c r="B63" s="9">
+        <f>IF(ISNUMBER(B60),B6-B60,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="4" t="inlineStr">
         <is>
           <t>¿Con tu número de personas cubres costos?</t>
         </is>
       </c>
-      <c r="B53" s="13">
-        <f>IF(ISNUMBER(B49),IF(B6&gt;=B49,"Sí, cubres costos","No, pierdes dinero"),"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="B64" s="13">
+        <f>IF(ISNUMBER(B60),IF(B6&gt;=B60,"Sí, cubres costos","No, pierdes dinero"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
         <is>
           <t>PRECIO DEL CUPO SEGÚN EL MARGEN QUE QUIERAS</t>
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="16" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="17" t="inlineStr">
         <is>
           <t>Margen</t>
         </is>
       </c>
-      <c r="B56" s="16" t="inlineStr">
+      <c r="B67" s="17" t="inlineStr">
         <is>
           <t>Precio del cupo</t>
         </is>
       </c>
-      <c r="C56" s="16" t="inlineStr">
+      <c r="C67" s="17" t="inlineStr">
         <is>
           <t>Ganancia total</t>
         </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="17" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B57" s="9">
-        <f>IF(1-$B$9-A57&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A57))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C57" s="9">
-        <f>IF(ISNUMBER(B57),B57*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="17" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B58" s="9">
-        <f>IF(1-$B$9-A58&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A58))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C58" s="9">
-        <f>IF(ISNUMBER(B58),B58*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="17" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="B59" s="9">
-        <f>IF(1-$B$9-A59&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A59))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C59" s="9">
-        <f>IF(ISNUMBER(B59),B59*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="17" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B60" s="9">
-        <f>IF(1-$B$9-A60&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A60))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="C60" s="9">
-        <f>IF(ISNUMBER(B60),B60*$B$6*(1-$B$9)-$B$33,"")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="3" t="inlineStr">
-        <is>
-          <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>Personas</t>
-        </is>
-      </c>
-      <c r="B63" s="16" t="inlineStr">
-        <is>
-          <t>Ingresos</t>
-        </is>
-      </c>
-      <c r="C63" s="16" t="inlineStr">
-        <is>
-          <t>Costo total</t>
-        </is>
-      </c>
-      <c r="D63" s="16" t="inlineStr">
-        <is>
-          <t>Ganancia</t>
-        </is>
-      </c>
-      <c r="E63" s="16" t="inlineStr">
-        <is>
-          <t>Margen</t>
-        </is>
-      </c>
-      <c r="F63" s="16" t="inlineStr">
-        <is>
-          <t>Precio para tu margen</t>
-        </is>
-      </c>
-      <c r="G63" s="16" t="inlineStr">
-        <is>
-          <t>¿Cubre costos?</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="B64" s="9">
-        <f>$B$7*A64</f>
-        <v/>
-      </c>
-      <c r="C64" s="9">
-        <f>($B$29+$B$28*A64)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D64" s="19">
-        <f>B64*(1-$B$9)-C64</f>
-        <v/>
-      </c>
-      <c r="E64" s="20">
-        <f>IF(B64&gt;0,D64/B64,0)</f>
-        <v/>
-      </c>
-      <c r="F64" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C64/(A64*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G64" s="13">
-        <f>IF(D64&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="B65" s="9">
-        <f>$B$7*A65</f>
-        <v/>
-      </c>
-      <c r="C65" s="9">
-        <f>($B$29+$B$28*A65)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D65" s="19">
-        <f>B65*(1-$B$9)-C65</f>
-        <v/>
-      </c>
-      <c r="E65" s="20">
-        <f>IF(B65&gt;0,D65/B65,0)</f>
-        <v/>
-      </c>
-      <c r="F65" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C65/(A65*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G65" s="13">
-        <f>IF(D65&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="B66" s="9">
-        <f>$B$7*A66</f>
-        <v/>
-      </c>
-      <c r="C66" s="9">
-        <f>($B$29+$B$28*A66)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D66" s="19">
-        <f>B66*(1-$B$9)-C66</f>
-        <v/>
-      </c>
-      <c r="E66" s="20">
-        <f>IF(B66&gt;0,D66/B66,0)</f>
-        <v/>
-      </c>
-      <c r="F66" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C66/(A66*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G66" s="13">
-        <f>IF(D66&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="18" t="n">
-        <v>11</v>
-      </c>
-      <c r="B67" s="9">
-        <f>$B$7*A67</f>
-        <v/>
-      </c>
-      <c r="C67" s="9">
-        <f>($B$29+$B$28*A67)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D67" s="19">
-        <f>B67*(1-$B$9)-C67</f>
-        <v/>
-      </c>
-      <c r="E67" s="20">
-        <f>IF(B67&gt;0,D67/B67,0)</f>
-        <v/>
-      </c>
-      <c r="F67" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C67/(A67*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G67" s="13">
-        <f>IF(D67&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="18" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B68" s="8">
+        <f>IF(1-$B$9-A68&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A68))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C68" s="8">
+        <f>IF(ISNUMBER(B68),B68*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="18" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B69" s="8">
+        <f>IF(1-$B$9-A69&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A69))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C69" s="8">
+        <f>IF(ISNUMBER(B69),B69*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="B70" s="8">
+        <f>IF(1-$B$9-A70&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A70))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C70" s="8">
+        <f>IF(ISNUMBER(B70),B70*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="18" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="B71" s="8">
+        <f>IF(1-$B$9-A71&lt;=0,"",ROUNDUP($B$33/($B$6*(1-$B$9-A71))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="C71" s="8">
+        <f>IF(ISNUMBER(B71),B71*$B$6*(1-$B$9)-$B$33,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>SI CAMBIA EL NÚMERO DE PERSONAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="17" t="inlineStr">
+        <is>
+          <t>Personas</t>
+        </is>
+      </c>
+      <c r="B74" s="17" t="inlineStr">
+        <is>
+          <t>Ingresos</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>Costo total</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="inlineStr">
+        <is>
+          <t>Ganancia</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="inlineStr">
+        <is>
+          <t>Margen</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>Precio para tu margen</t>
+        </is>
+      </c>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>¿Cubre costos?</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="B75" s="8">
+        <f>$B$7*A75</f>
+        <v/>
+      </c>
+      <c r="C75" s="8">
+        <f>($B$29+$B$28*A75)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D75" s="20">
+        <f>B75*(1-$B$9)-C75</f>
+        <v/>
+      </c>
+      <c r="E75" s="14">
+        <f>IF(B75&gt;0,D75/B75,0)</f>
+        <v/>
+      </c>
+      <c r="F75" s="8">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C75/(A75*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G75" s="13">
+        <f>IF(D75&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="19" t="n">
+        <v>8</v>
+      </c>
+      <c r="B76" s="8">
+        <f>$B$7*A76</f>
+        <v/>
+      </c>
+      <c r="C76" s="8">
+        <f>($B$29+$B$28*A76)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D76" s="20">
+        <f>B76*(1-$B$9)-C76</f>
+        <v/>
+      </c>
+      <c r="E76" s="14">
+        <f>IF(B76&gt;0,D76/B76,0)</f>
+        <v/>
+      </c>
+      <c r="F76" s="8">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C76/(A76*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G76" s="13">
+        <f>IF(D76&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="19" t="n">
+        <v>10</v>
+      </c>
+      <c r="B77" s="8">
+        <f>$B$7*A77</f>
+        <v/>
+      </c>
+      <c r="C77" s="8">
+        <f>($B$29+$B$28*A77)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D77" s="20">
+        <f>B77*(1-$B$9)-C77</f>
+        <v/>
+      </c>
+      <c r="E77" s="14">
+        <f>IF(B77&gt;0,D77/B77,0)</f>
+        <v/>
+      </c>
+      <c r="F77" s="8">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C77/(A77*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G77" s="13">
+        <f>IF(D77&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="19" t="n">
+        <v>11</v>
+      </c>
+      <c r="B78" s="8">
+        <f>$B$7*A78</f>
+        <v/>
+      </c>
+      <c r="C78" s="8">
+        <f>($B$29+$B$28*A78)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D78" s="20">
+        <f>B78*(1-$B$9)-C78</f>
+        <v/>
+      </c>
+      <c r="E78" s="14">
+        <f>IF(B78&gt;0,D78/B78,0)</f>
+        <v/>
+      </c>
+      <c r="F78" s="8">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C78/(A78*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G78" s="13">
+        <f>IF(D78&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="19" t="n">
         <v>12</v>
       </c>
-      <c r="B68" s="9">
-        <f>$B$7*A68</f>
-        <v/>
-      </c>
-      <c r="C68" s="9">
-        <f>($B$29+$B$28*A68)*(1+$B$10)+$B$24</f>
-        <v/>
-      </c>
-      <c r="D68" s="19">
-        <f>B68*(1-$B$9)-C68</f>
-        <v/>
-      </c>
-      <c r="E68" s="20">
-        <f>IF(B68&gt;0,D68/B68,0)</f>
-        <v/>
-      </c>
-      <c r="F68" s="9">
-        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C68/(A68*(1-$B$9-$B$8))/5000,0)*5000)</f>
-        <v/>
-      </c>
-      <c r="G68" s="13">
-        <f>IF(D68&gt;=0,"Sí","No: pierdes")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="B79" s="8">
+        <f>$B$7*A79</f>
+        <v/>
+      </c>
+      <c r="C79" s="8">
+        <f>($B$29+$B$28*A79)*(1+$B$10)+$B$24</f>
+        <v/>
+      </c>
+      <c r="D79" s="20">
+        <f>B79*(1-$B$9)-C79</f>
+        <v/>
+      </c>
+      <c r="E79" s="14">
+        <f>IF(B79&gt;0,D79/B79,0)</f>
+        <v/>
+      </c>
+      <c r="F79" s="8">
+        <f>IF(1-$B$9-$B$8&lt;=0,"",ROUNDUP(C79/(A79*(1-$B$9-$B$8))/5000,0)*5000)</f>
+        <v/>
+      </c>
+      <c r="G79" s="13">
+        <f>IF(D79&gt;=0,"Sí","No: pierdes")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
         <is>
           <t>Nota: pinceles, esponjas y delantales se compran una vez; en los próximos talleres el costo fijo baja. Los datos marcados ESTIMADO no son cotizaciones reales.</t>
         </is>
       </c>
     </row>
-    <row r="71">
-      <c r="A71" s="2" t="inlineStr">
-        <is>
-          <t>El restaurante pone lugar, aperitivos y vino; por eso esos costos no aparecen aquí.</t>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>El restaurante pone lugar, aperitivos y vino; el pago que acuerdes se descuenta de tu ganancia. Los escenarios usan el mismo pago.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A70:G70"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A55:G55"/>
-    <mergeCell ref="A48:G48"/>
+  <mergeCells count="12">
+    <mergeCell ref="A66:G66"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A53:G53"/>
     <mergeCell ref="A26:G26"/>
-    <mergeCell ref="A62:G62"/>
+    <mergeCell ref="A2:G2"/>
     <mergeCell ref="A42:G42"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A59:G59"/>
+    <mergeCell ref="A81:G81"/>
+    <mergeCell ref="A73:G73"/>
+    <mergeCell ref="A82:G82"/>
     <mergeCell ref="A5:G5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Taller de cerámica: lista de compras de materiales ($250.000) y delantales a $20.000
Lista para 15 personas sin pigmentos: papel acuarela para ensayar, lápices,
pinceles, esponjas y mesa, con colchón. La cuenta queda con materiales
$250.000 y 15 delantales a $20.000.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0143Qo8ykWtKoT2mCgP12s2c
</commit_message>
<xml_diff>
--- a/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
+++ b/docs/sesion-2026-10-02/cotizacion-taller-ceramica.xlsx
@@ -67,7 +67,7 @@
     <t xml:space="preserve">Pigmentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Pinceles, esponjas y materiales</t>
+    <t xml:space="preserve">Materiales (lista de compras)</t>
   </si>
   <si>
     <t xml:space="preserve">Delantales</t>
@@ -714,26 +714,27 @@
         <v>1</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>200000</v>
+        <v>250000</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">B15*C15</f>
-        <v>200000</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="5" t="n">
-        <v>1</v>
+      <c r="B16" s="10" t="n">
+        <f aca="false">B5</f>
+        <v>15</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>120000</v>
+        <v>20000</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">B16*C16</f>
-        <v>120000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -819,7 +820,7 @@
       </c>
       <c r="D22" s="13" t="n">
         <f aca="false">SUM(D11:D21)</f>
-        <v>2353800</v>
+        <v>2583800</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -845,7 +846,7 @@
       </c>
       <c r="B26" s="11" t="n">
         <f aca="false">D22</f>
-        <v>2353800</v>
+        <v>2583800</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -854,7 +855,7 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">B25-B26</f>
-        <v>1096200</v>
+        <v>866200</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -863,7 +864,7 @@
       </c>
       <c r="B28" s="11" t="n">
         <f aca="false">B27/B5</f>
-        <v>73080</v>
+        <v>57746.6666666667</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -872,7 +873,7 @@
       </c>
       <c r="B29" s="15" t="n">
         <f aca="false">IF(B25&gt;0,B27/B25,0)</f>
-        <v>0.317739130434783</v>
+        <v>0.251072463768116</v>
       </c>
     </row>
   </sheetData>

</xml_diff>